<commit_message>
Added Save to BD function for Clubs
</commit_message>
<xml_diff>
--- a/olympic_simulator/media/simulacion_AFC Challenge League_1880.xlsx
+++ b/olympic_simulator/media/simulacion_AFC Challenge League_1880.xlsx
@@ -485,29 +485,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="C3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
         <v>18</v>
       </c>
-      <c r="D3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>17</v>
-      </c>
       <c r="H3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" t="n">
         <v>8</v>
-      </c>
-      <c r="I3" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -516,29 +516,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I4" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -547,29 +547,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I5" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -578,29 +578,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I6" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="7">
@@ -609,29 +609,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H7" t="n">
         <v>14</v>
       </c>
       <c r="I7" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="10">
@@ -666,88 +666,88 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -756,102 +756,102 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -864,70 +864,70 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="C25" t="n">
         <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>2</v>
@@ -936,52 +936,52 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
         <v>1</v>
@@ -990,34 +990,34 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
         <v>3</v>
@@ -1097,29 +1097,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1144,13 +1144,13 @@
         <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H4" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -1159,29 +1159,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
+        <v>11</v>
+      </c>
+      <c r="H5" t="n">
         <v>12</v>
       </c>
-      <c r="H5" t="n">
-        <v>10</v>
-      </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="6">
@@ -1190,26 +1190,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I6" t="n">
         <v>-6</v>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1237,13 +1237,13 @@
         <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I7" t="n">
-        <v>-12</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="10">
@@ -1278,16 +1278,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -1296,232 +1296,232 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -1530,88 +1530,88 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>2</v>
@@ -1620,19 +1620,19 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1709,29 +1709,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1759,10 +1759,10 @@
         <v>7</v>
       </c>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="5">
@@ -1771,29 +1771,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Navua FC</t>
+          <t>Wolmido SC</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I5" t="n">
-        <v>-3</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="6">
@@ -1802,29 +1802,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FC Chitwan</t>
+          <t>Brera Ilch FC</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I6" t="n">
-        <v>-1</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="9">
@@ -1859,30 +1859,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>Wolmido SC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FC Chitwan</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Navua FC</t>
+          <t>Brera Ilch FC</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1895,16 +1895,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>Wolmido SC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Navua FC</t>
+          <t>Brera Ilch FC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -1913,34 +1913,34 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FC Chitwan</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>Wolmido SC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>2</v>
@@ -1949,88 +1949,88 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Navua FC</t>
+          <t>Brera Ilch FC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FC Chitwan</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FC Chitwan</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>Wolmido SC</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Navua FC</t>
+          <t>Brera Ilch FC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Navua FC</t>
+          <t>Brera Ilch FC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>Wolmido SC</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FC Chitwan</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -2039,16 +2039,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>Wolmido SC</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -2057,19 +2057,19 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FC Chitwan</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Navua FC</t>
+          <t>Brera Ilch FC</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2146,26 +2146,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" t="n">
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I3" t="n">
         <v>3</v>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -2193,13 +2193,13 @@
         <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="5">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Royal Thimphu College FC</t>
+          <t>Bangladesh Police FC</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -2224,13 +2224,13 @@
         <v>2</v>
       </c>
       <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
         <v>8</v>
       </c>
-      <c r="H5" t="n">
-        <v>7</v>
-      </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -2239,29 +2239,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AS Pueu</t>
+          <t>FK Kopetdag Asgabat</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H6" t="n">
         <v>10</v>
       </c>
       <c r="I6" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="9">
@@ -2296,34 +2296,34 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AS Pueu</t>
+          <t>FK Kopetdag Asgabat</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Bangladesh Police FC</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Royal Thimphu College FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -2332,12 +2332,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AS Pueu</t>
+          <t>FK Kopetdag Asgabat</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2350,34 +2350,34 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Bangladesh Police FC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Royal Thimphu College FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AS Pueu</t>
+          <t>FK Kopetdag Asgabat</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Royal Thimphu College FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -2386,127 +2386,127 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Bangladesh Police FC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Bangladesh Police FC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AS Pueu</t>
+          <t>FK Kopetdag Asgabat</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Royal Thimphu College FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AS Pueu</t>
+          <t>FK Kopetdag Asgabat</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Royal Thimphu College FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Bangladesh Police FC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Royal Thimphu College FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AS Pueu</t>
+          <t>FK Kopetdag Asgabat</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Bangladesh Police FC</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -2599,13 +2599,13 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -2630,13 +2630,13 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -2645,29 +2645,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2676,29 +2676,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="7">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -2723,10 +2723,10 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
         <v>-1</v>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -2757,10 +2757,10 @@
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="9">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -2816,13 +2816,13 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
         <v>4</v>
       </c>
       <c r="I10" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="13">
@@ -2857,106 +2857,106 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -2965,34 +2965,34 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
         <v>2</v>
@@ -3072,29 +3072,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FC Neftchi Kochkor Ata</t>
+          <t>FC Bishkek City</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -3103,29 +3103,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ryomyong SC</t>
+          <t>Al Ittihad Ahli SC</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H4" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Al Jaish SC</t>
+          <t>Nadi FC</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -3150,13 +3150,13 @@
         <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H5" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3165,29 +3165,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ashgabat FK</t>
+          <t>AS Temanava</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H6" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="7">
@@ -3196,29 +3196,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AC de Ultramar</t>
+          <t>Port Moresby Strikers</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G7" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H7" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hekari United</t>
+          <t>Butwal Lumbini FC</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -3240,16 +3240,16 @@
         <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H8" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I8" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hunters FC</t>
+          <t>Dagon Port FC</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -3271,16 +3271,16 @@
         <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H9" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I9" t="n">
-        <v>-5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="10">
@@ -3289,26 +3289,26 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ISPE FC</t>
+          <t>Master FC</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I10" t="n">
         <v>2</v>
@@ -3320,29 +3320,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Boeung Ket FC</t>
+          <t>Kirivong Sok Sen Chey FC</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
         <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>4</v>
       </c>
       <c r="G11" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H11" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I11" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="12">
@@ -3351,29 +3351,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Master FC</t>
+          <t>Benfica de Macau FC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H12" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I12" t="n">
-        <v>-1</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="13">
@@ -3382,29 +3382,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Royal Thimphu College FC</t>
+          <t>Hang Yuan FC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H13" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="14">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cheng Fung</t>
+          <t>Bangladesh Police FC</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -3426,16 +3426,16 @@
         <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
         <v>10</v>
       </c>
       <c r="H14" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I14" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -3444,29 +3444,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dhaka Wanderers</t>
+          <t>FK Kopetdag Asgabat</t>
         </is>
       </c>
       <c r="C15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" t="n">
         <v>8</v>
       </c>
-      <c r="D15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" t="n">
-        <v>4</v>
-      </c>
-      <c r="G15" t="n">
-        <v>12</v>
-      </c>
       <c r="H15" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I15" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="16">
@@ -3475,17 +3475,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AC Taipei</t>
+          <t>Samtse FC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>4</v>
@@ -3506,29 +3506,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Navua FC</t>
+          <t>Wolmido SC</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I17" t="n">
-        <v>-3</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="18">
@@ -3537,29 +3537,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FC Chitwan</t>
+          <t>Lun Bawang FC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I18" t="n">
-        <v>-1</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="19">
@@ -3568,26 +3568,26 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AS Pueu</t>
+          <t>Brera Ilch FC</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G19" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H19" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I19" t="n">
         <v>-4</v>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kota Ranger FC</t>
+          <t>FC Porto Taibesse</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -3615,13 +3615,13 @@
         <v>6</v>
       </c>
       <c r="G20" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I20" t="n">
-        <v>-12</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="23">

</xml_diff>